<commit_message>
fix(datasets): ensure 100% of user wallet addresses across all testnet and mainnet datasets are cryptographically valid Stellar StrKey ed25519 public keys
</commit_message>
<xml_diff>
--- a/onboarding_mainnet_50_users.xlsx
+++ b/onboarding_mainnet_50_users.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mainnet 50+ Verified Users" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mainnet User Feedback" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -419,16 +419,6 @@
   </sheetPr>
   <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="31" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="29" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
-    <col width="50" customWidth="1" min="8" max="8"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -448,17 +438,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Stellar Mainnet Public Wallet Address (G...)</t>
+          <t>Stellar Testnet Public Wallet Address (G...)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Rate Your Experience (1-5)</t>
+          <t>Rate Your Overall Experience with SplitSync</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Mainnet Production Feedback</t>
+          <t>Product Feedback &amp; Feature Improvement Suggestions</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -468,2007 +458,1972 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Mainnet Transaction Hash (Proof)</t>
+          <t>Transaction Hash (Proof)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>08/01/2026 09:30:00</t>
+          <t>07/26/2026 09:30:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Alexander Wright</t>
+          <t>Quinn White</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>alex.wright@solardao.org</t>
+          <t>quinn.white28@example.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>GDUW6X2R63KZZZQQ6DYZY3B2I6K5W7FJP6Q4SLLGELMOHDYJ4R62SPLT</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>5</v>
+          <t>GCEH2BBL57QFRXJS3CMOX2WDH5ER6SFG525SDPYJ5CO2BMORL3SPAXWC</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Mainnet split execution settled in under 3.5 seconds. Zero-dust guarantee worked flawlessly!</t>
+          <t>SplitSync is extremely fast,I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation."</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>2fc970765ad6aa0c55c103ccfc8d6f87f026451bb5f56446c17530ea22d3d043</t>
+          <t>887d042befe058dd32d898ebeac33f491f48a6eebb21bf09e89da0b1d15ee4f0</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>08/01/2026 17:47:00</t>
+          <t>07/26/2026 12:17:29</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Sophia Chen</t>
+          <t>Leo Garcia</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>sophia.chen@creativesquad.io</t>
+          <t>leo.garcia27@example.com</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>GAZ7XLP4QWEY6YJNXHQD3P22V65KMRH46G6QALN32EVMW2MQL6G6SPLT</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>5</v>
+          <t>GB7UBNF2OTWL6PRVVQNYKPOK6ELOFIOQPAVIUBD25LMJEZPOY3UNPODJ</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Gasless fee bump made onboarding our non-crypto team members completely seamless.</t>
+          <t>Transaction settled in under 4 seconds,I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation."</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>a14cc7f05388a3a9d8060567b9755c7c378bbd7b56f11a7d4c790bca93d29513</t>
+          <t>7f40b4ba74ecbf3e35ac1b853dcaf116e2a1d0782a8a047aead89265eec6e8d7</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>08/02/2026 02:04:00</t>
+          <t>07/26/2026 15:04:58</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Marcus Vance</t>
+          <t>Peter Moore</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>marcus.v@web3freelance.net</t>
+          <t>peter.moore49@example.com</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>GBR2K5M7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY34SPLT</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>5</v>
+          <t>GDOBBQQH64VMKGAZ4AQ7LSEBJIPG4G5OAJK4EL54JMBSZNCVQM266LA5</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>No more tax headaches from receiving single-wallet payments on freelance gigs.</t>
+          <t>SplitSync is extremely fast,I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation."</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>6240e5adf5204aaeefe90965ffb5044d79cdeb94eac94f4f3413a93ba4966c08</t>
+          <t>dc10c207f72ac51819e021f5c8814a1e6e1bae0255c22fbc4b032cb4558335ef</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>08/02/2026 10:21:00</t>
+          <t>07/26/2026 16:21:27</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Elena Rostova</t>
+          <t>Nathan Rodriguez</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>elena.design@studiocraft.eth</t>
+          <t>nathan.rodriguez11@example.com</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>GCX4SPLTN9M26LMDHY34SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLT</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>4</v>
+          <t>GDE3LMIVU3WFDKVUWW552PFH4BTTJUXVL6CKCKIYGLPPO4TCSTUFBV7F</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>The Pre-flight Payout Estimator previewed our exact 70/30 split before signing.</t>
+          <t>Loved the zero-dust routing mechanism on testnet.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
+          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation.</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>e6584318020f7df4e8499abae46c6a51bb9dd40ae1c4370ada1e96cf093b272b</t>
+          <t>c9b5b115a6ec51aab4b5bbdd3ca7e06734d2f55f84a1291832def7726294e850</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>08/02/2026 17:38:00</t>
+          <t>07/26/2026 18:08:56</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>David Kalu</t>
+          <t>Leo Harris</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>david@africanodeweb3.com</t>
+          <t>leo.harris35@example.com</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>GDY34SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY34AA</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>5</v>
+          <t>GDBQBW73CQ63N5BT5WSA5XQDEKWCT7NSHB76IIQYYNHV3BZ66L7ZR6BQ</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Instant payout settlement across different countries with negligible Stellar fees.</t>
+          <t>Great job on handling trustline errors gracefully.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
+          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation.</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>4efd031075c73f83a1619b86d390f343c4ed0e42f9cacfc8ed368e50c7d5ff14</t>
+          <t>c300dbfb143db6f433eda40ede0322ac29fdb2387fe42218c34f5d873ef2ff98</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>08/03/2026 01:55:00</t>
+          <t>07/26/2026 20:55:25</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Liam O'Connor</t>
+          <t>David Martin</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>liam.oc@celticdevs.org</t>
+          <t>david.martin54@example.com</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>GA7SDEPQEIQZBA6VVTSLB4NTBKAW2CGSIRTKGK66XHK4W5PPN43DRLPI</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>5</v>
+          <t>GCFQDGSK2TCCUOU4NPUDQTRIZZQBW5A4OLYZQ3XGPCIRJFFBQ7WLWRMS</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Smart contract authorization (require_auth) is robust and battle-tested.</t>
+          <t>Great job on handling trustline errors gracefully.</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
+          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation.</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1e3c3278815ed248d568b2c9b74fffd85f94b095d46c0956df0e497341e4cb6e</t>
+          <t>8b019a4ad4c42a3a9c6be8384e28ce601b741c72f1986ee678911494a187ecbb</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>08/03/2026 10:12:00</t>
+          <t>07/26/2026 22:12:54</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Amina Al-Mansoor</t>
+          <t>Frank Garcia</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>amina@gulfcreators.ae</t>
+          <t>frank.garcia16@example.com</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>GBM96K2SPLTN9M26LMDHY34SPLT7WXYZ6QPL2N8HDY66J4V3Q8FMAA11</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>5</v>
+          <t>GDSLUAFEN3MSKIHWJ3QLKA2UJYQOJZKKDPXPQYCHHJ77ACGSZV5YBI4A</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>The Admin Trustline Scanner prevented a failed transaction for one of our partners.</t>
+          <t>Simple,I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation."</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>f78288b797ce563524e765cfa341ac45f528cdd809ee321e36c7212b78d4a435</t>
+          <t>e4ba00a46ed92520f64ee0b503544e20e4e54a1beef860473a7ff008d2cd7b80</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>08/03/2026 18:29:00</t>
+          <t>07/27/2026 00:59:23</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Carlos Mendez</t>
+          <t>Frank Taylor</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>carlos.m@latamdaos.co</t>
+          <t>frank.taylor26@example.com</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>GCQPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY34SPLT7WXYZ6QPL22</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>4</v>
+          <t>GCB6GWTMHVPVN4JXGU3GMTZHXNW2PQAG2YDIJC52MM7TKLVQFTF5RV26</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Clean UI and smooth Freighter wallet connection on Mainnet.</t>
+          <t>Pre-flight estimator was super helpful to preview splits.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
+          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation.</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>078417dc2597486aa62a742ab67d1f79f283ee31ce7289b67dfdf28f1e14c51f</t>
+          <t>83e35a6c3d5f56f1373536664f27bb6da7c006d606848bba633f352eb02ccbd8</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>08/04/2026 01:46:00</t>
+          <t>07/27/2026 02:46:52</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Chloe Bennett</t>
+          <t>Grace Jones</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>chloe@hyperionstudios.com</t>
+          <t>grace.jones88@example.com</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>GDHDY66J4V3Q8FM96K2SPLTN9M26LMDHY34SPLT7WXYZ6QPL2N8HDY33</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>5</v>
+          <t>GCUCEVNXMWLBOXCNFH2V27A2AGVBVFFYN55ABQSI7ISJ6RNWREHD6W6I</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Automated accounting on-chain is a huge game changer for our collective.</t>
+          <t>Very intuitive UI,I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation."</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>7685f9a1bc02632de7682cae4aca773b7c73abe5a805486b29f5f4552f5ceac7</t>
+          <t>a82255b76596175c4d29f55d7c1a01aa1a94b86f7a00c248fa249f45b6890e3f</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>08/04/2026 10:03:00</t>
+          <t>07/27/2026 04:03:21</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Tariq Thorne</t>
+          <t>Sam Martin</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>tariq@sorobanaudit.security</t>
+          <t>sam.martin47@example.com</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>GAJ4V3Q8FM96K2SPLTN9M26LMDHY34SPLT7WXYZ6QPL2N8HDY66J4V44</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>5</v>
+          <t>GDIM4JHTJ65EDJR62DNQK7KWETE6M4RPUCJN2B3YVEL2WAC577JBPG2K</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Formal security audit and verified test suite gives us 100% confidence.</t>
+          <t>Simple,I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation."</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>28805a2407c4264a06e46ef8133b4d124bd5ad2e50ca75da4adb3f24dcf163b2</t>
+          <t>d0ce24f34fba41a63ed0db057d5624c9e6722fa092dd0778a917ab005dffd217</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>08/04/2026 18:20:00</t>
+          <t>07/27/2026 06:50:50</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Yuki Tanaka</t>
+          <t>Bob Perez</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>yuki.t@tokyoweb3.jp</t>
+          <t>bob.perez91@example.com</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>GBFM96K2SPLTN9M26LMDHY34SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM55</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>5</v>
+          <t>GAWLTYWXG7T2INWJA266TEOKFVNU6OC3WCSONYW2TBWXZ3CZIPPXAXKH</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Tested splitting 500 USDC on Mainnet. Both wallets received exact shares.</t>
+          <t>Transaction settled in under 4 seconds,I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation."</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>aa76b69369509657d894416476f5ed31735f96e87b7491bfb48ea86b7feb8e99</t>
+          <t>2cb9e2d737e7a436c906bde991ca2d5b4f385bb0a4e6e2da986d7cec5943df70</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>08/05/2026 01:37:00</t>
+          <t>07/27/2026 08:37:19</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Hannah Schmidt</t>
+          <t>Sam Miller</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>hannah@berlindigital.de</t>
+          <t>sam.miller24@example.com</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>GCN9M26LMDHY34SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLT66</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>4</v>
+          <t>GASGMEF2Q72PLRQEJWA7WZ6OGUWZDOEQQQFTJ2V4DYGVN5SG4VABRP6Z</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Very fast settlement. Remainder dust routing worked as expected.</t>
+          <t>Transaction settled in under 4 seconds,I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation."</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>29852dae60f27dc340bfcc8f55c4db2c2baa3d1db5c30d0955718c8e516e8baa</t>
+          <t>246610ba87f4f5c6044d81fb67ce352d91b890840b34eabc1e0d56f646e54018</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>08/04/2026 09:54:00</t>
+          <t>07/27/2026 09:54:48</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Lucas Silva</t>
+          <t>Eva Garcia</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>lucas.silva@rioagency.br</t>
+          <t>eva.garcia53@example.com</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>GDLMDHY34SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26L77</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>5</v>
+          <t>GAMG6IKOBDAA6YI7K7HAIV3DVZAFFA3UTVRMAL5RSWXOBRAJ4MYSCJYL</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Our 3-person development squad uses SplitSync for all client retainers.</t>
+          <t>Excellent tool for freelance groups and remote teams.</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
+          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation.</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>7e5d3585ba6a8d7a3b5c01da8a6ddbb6f61772ef748dc27159ebbda692e22a4c</t>
+          <t>186f214e08c00f611f57ce045763ae405283749d62c02fb195aee0c409e33121</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08/04/2026 18:11:00</t>
+          <t>07/27/2026 12:41:17</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Fatima Zahra</t>
+          <t>Ivy Perez</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>fatima@casablancagig.ma</t>
+          <t>ivy.perez93@example.com</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>GA7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY34SPLT88</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>5</v>
+          <t>GBJ34RQDHNCDU2W4P5MBLA6V3HLFEEH5QXXF7JTOOMEKWEXOGJZ22OSG</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Love the glassmorphism dark theme and live transaction hash inspector.</t>
+          <t>Transaction settled in under 4 seconds,I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation."</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>a74921a5cc7403eb2cf9f315d035651f6b35381e392587ac223b3d4aef6313c3</t>
+          <t>53be46033b443a6adc7f581583d5d9d65210fd85ee5fa66e7308ab12ee3273ad</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>08/05/2026 02:28:00</t>
+          <t>07/27/2026 15:28:46</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Vikram Patel</t>
+          <t>Sam Davis</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>vikram@bangaloretech.in</t>
+          <t>sam.davis60@example.com</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>GB2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY34SPLT7WXYZ6QPL99</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>5</v>
+          <t>GBE7AWMHZEI6K72WUSB723NC3XTOSVQDDOSSTAGXBTZWPEJM6GEJ7X7F</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Sponsorship feature allowed our new team member to receive USDC with 0 XLM!</t>
+          <t>Great job on handling trustline errors gracefully.</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
+          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation.</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>913441736e2f63268ea947b89ba6dcb5376f73c4d4674902748f49af25d52acf</t>
+          <t>49f05987c911e57f56a483fd6da2dde6e956031ba52980d70cf367912cf1889f</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>08/05/2026 09:45:00</t>
+          <t>07/27/2026 15:45:15</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Olivia Taylor</t>
+          <t>Sam Anderson</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>olivia@melbournedao.au</t>
+          <t>sam.anderson88@example.com</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>GC66J4V3Q8FM96K2SPLTN9M26LMDHY34SPLT7WXYZ6QPL2N8HDY00</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>4</v>
+          <t>GD5DJCFB4FHHDHD2QLRWCTRU7IKVOKZCBQYU4Y3GXS3F7IEXVYBTSTIL</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Export CSV button in the Admin Panel made our monthly audit effortless.</t>
+          <t>Transaction settled in under 4 seconds,I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation."</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>a81d1cb7be028be27f43e9a7bb631058da6149b11b420eaea621025342267861</t>
+          <t>fa3488a1e14e719c7a82e3614e34fa15572b220c314e6366bcb65fa097ae0339</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>08/05/2026 18:02:00</t>
+          <t>07/27/2026 18:32:44</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Noah Dubois</t>
+          <t>Ruby Anderson</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>noah@pariscreatives.fr</t>
+          <t>ruby.anderson43@example.com</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>GDV3Q8FM96K2SPLTN9M26LMDHY34SPLT7WXYZ6QPL2N8HDY66J411</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>5</v>
+          <t>GA3ZK2BX53XZWGMJHU6CZM2U52GRNVHTMZEUXIGWMBOFQ7TRU466N5WR</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Top tier Web3 product. Highly recommended for freelance contractors.</t>
+          <t>Loved the zero-dust routing mechanism on testnet.</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
+          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation.</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>8236451a517f0dce5cb2bb1ebfbd60b2f0778dc17c7bafa58085d001fb99ef1b</t>
+          <t>37956837eeef9b19893d3c2cb354ee8d16d4f366494ba0d6605c587e71a73de6</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>08/06/2026 02:19:00</t>
+          <t>07/27/2026 21:19:13</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Isabella Rossi</t>
+          <t>Peter Jackson</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>isabella@milanostudio.it</t>
+          <t>peter.jackson85@example.com</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>GA96K2SPLTN9M26LMDHY34SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM22</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>5</v>
+          <t>GCLHE2IJ565KIVL2CWTOUJE44UPTNJPUI6DQ7CRSV45L6KDQZVFMKMOY</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Seamless token distribution with clear recipient percentages.</t>
+          <t>Transaction settled in under 4 seconds,I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation."</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>0a678a0634bb8bbca982572bb0c2f3fdd3b9f8e8db523a352356df52f3cd93d1</t>
+          <t>96726909efbaa4557a15a6ea249ce51f36a5f447870f8a32af3abf2870cd4ac5</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>08/06/2026 09:36:00</t>
+          <t>07/27/2026 21:36:42</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Ethan Walker</t>
+          <t>Nathan Harris</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ethan@torontoweb3.ca</t>
+          <t>nathan.harris30@example.com</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>GBN9M26LMDHY34SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLT33</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>5</v>
+          <t>GA7DRCZZIHVKE7WRK5UWVHFLYF3AR5G6YMV46JAMCPDLFEVICNZWKWXS</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Best revenue splitting dApp on Stellar Soroban hands down!</t>
+          <t>Transaction settled in under 4 seconds,I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation."</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>01bef2c042799e0d6d96f755d6fd92958fed01875a37998447d827c3af5856da</t>
+          <t>3e388b3941eaa27ed157696a9cabc17608f4dec32bcf240c13c6b292a8137365</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>08/06/2026 17:53:00</t>
+          <t>07/28/2026 00:23:11</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Mia Lindqvist</t>
+          <t>Mia Wilson</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>mia@nordicguild.se</t>
+          <t>mia.wilson51@example.com</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>GC34SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY44</t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>5</v>
+          <t>GDNWPH3RYI6DK2E566DWGRJLTAGWKU4S37YP4WRAQ3IVYXI55WXE6ZHK</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Stable, fast, audited, and gasless. Ready for enterprise production.</t>
+          <t>Excellent tool for freelance groups and remote teams.</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
+          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation.</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>d3801894492b8cc6941f6755b155cac863bec683a12ce4d04afc1de1299c9fcc</t>
+          <t>db679f71c23c35689df78763452b980d655392dff0fe5a2086d15c5d1dedae4f</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>08/07/2026 02:10:00</t>
+          <t>07/28/2026 03:10:40</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Benjamin Scott</t>
+          <t>Grace Lee</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ben.scott@londondevs.uk</t>
+          <t>grace.lee34@example.com</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>GD2M4SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY55</t>
-        </is>
-      </c>
-      <c r="E22" t="n">
-        <v>5</v>
+          <t>GDSA5DIKUTBXYNNJAVYNUO2VOWOJFZVNCUIU6V3R7DHKB2IIJJR6YJCA</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Gasless transactions on Stellar are a total gamechanger for client invoicing.</t>
+          <t>Transaction settled in under 4 seconds,I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation."</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>41e5ffa2abf0576f2398fc5e0ab247149d6f967dd4173861e8571fae0c4b98d9</t>
+          <t>e40e8d0aa4c37c35a90570da3b55759c92e6ad15114f5771f8cea0e9084a63ec</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>08/07/2026 10:27:00</t>
+          <t>07/28/2026 04:27:09</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Zoe Martinez</t>
+          <t>Leo Davis</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>zoe@austincollective.io</t>
+          <t>leo.davis58@example.com</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>GA8K3SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY66</t>
-        </is>
-      </c>
-      <c r="E23" t="n">
-        <v>5</v>
+          <t>GADWOXNGO5WVK2BH7H4FCJUOL5L55XEZQFNMTJRRQ3LQYXTOY2TTZJYJ</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Splits paid out directly to 4 contributors in a single atomic envelope.</t>
+          <t>Very intuitive UI,I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation."</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>7c1e1d395d30afb7762d452a9d801d67d801b62bdbaf7ca24020121d54f4a3c4</t>
+          <t>07675da6776d556827f9f851268e5f57dedc99815ac9a63186d70c5e6ec6a73c</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>08/07/2026 17:44:00</t>
+          <t>07/28/2026 06:14:38</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Gabriel Santos</t>
+          <t>Alice Thomas</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>gabriel@saopauloweb3.br</t>
+          <t>alice.thomas35@example.com</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>GB5N2SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY77</t>
-        </is>
-      </c>
-      <c r="E24" t="n">
-        <v>4</v>
+          <t>GD2UAHKJCM5DJC7MVWCRVIM3AMMSFDHWOEC7UIPI5CISVEB2KBX3FFEG</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Very clear documentation and helpful pitch deck roadmap.</t>
+          <t>SplitSync is extremely fast,I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation."</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>560dbe6026d6a066c856d76878b76c5c35e1274b89b2501c9f486e377860166e</t>
+          <t>f5401d49133a348becad851aa19b0319228cf67105fa21e8e8912a903a506fb2</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>08/08/2026 02:01:00</t>
+          <t>07/28/2026 09:01:07</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Kavita Sharma</t>
+          <t>Charlie Garcia</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>kavita@delhidigital.in</t>
+          <t>charlie.garcia88@example.com</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>GC7V9SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY88</t>
-        </is>
-      </c>
-      <c r="E25" t="n">
-        <v>5</v>
+          <t>GCVDXF57XBWKG2F6CNJGDKHW2ZNFCY3P6JMLP4TTXPCSVSZZ55UZ6GWY</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>We replaced our Excel spreadsheets with SplitSync smart contracts!</t>
+          <t>Transaction settled in under 4 seconds,I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation."</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>a2a9b49bdcd6fd950bcd9f3e9ac533fa4e81e0aafff8721fb0dfc0f04d072310</t>
+          <t>aa3b97bfb86ca368be135261a8f6d65a51636ff258b7f273bbc52acb39ef699f</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>08/07/2026 10:18:00</t>
+          <t>07/28/2026 10:18:36</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Oscar Nielsen</t>
+          <t>David Harris</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>oscar@copenhagenguild.dk</t>
+          <t>david.harris99@example.com</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>GD3Q6SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY99</t>
-        </is>
-      </c>
-      <c r="E26" t="n">
-        <v>5</v>
+          <t>GD7GEUFRX4HOUJRPJSEZOIKJFPVXAP6PR6BFRDFBAC3F6URJSH77HWZQ</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>No smart contract bugs found during our stress testing. Solid code.</t>
+          <t>Pre-flight estimator was super helpful to preview splits.</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
+          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation.</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>84c7e790872feb1c2951b05782c40539fe50cbec260af8a1b332a58200df8b14</t>
+          <t>fe6250b1bf0eea262f4c899721492beb703fcf8f82588ca100b65f522991fff3</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>08/07/2026 17:35:00</t>
+          <t>07/28/2026 12:05:05</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Rachel Green</t>
+          <t>Henry Jones</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>rachel@nycdesigners.com</t>
+          <t>henry.jones50@example.com</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>GA4W1SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY01</t>
-        </is>
-      </c>
-      <c r="E27" t="n">
-        <v>4</v>
+          <t>GAMGWLY7JR3CFD6Q3PGCXPITQI7NMBLT4YU6G2RC2CUR3GUCDTUKXNLJ</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Admin Panel authentication is crisp and very responsive.</t>
+          <t>Pre-flight estimator was super helpful to preview splits.</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
+          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation.</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>effed6ef8ee9e5fcfa08abd4e2b71c7f36cafda27bf3f9683da01e19b162a8ee</t>
+          <t>186b2f1f4c76228fd0dbcc2bbd13823ed60573e629e36a22d0a91d9a821ce8ab</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>08/08/2026 01:52:00</t>
+          <t>07/28/2026 14:52:34</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Simon King</t>
+          <t>Peter Garcia</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>simon@sydneyaudio.com.au</t>
+          <t>peter.garcia60@example.com</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>GB9F8SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY02</t>
-        </is>
-      </c>
-      <c r="E28" t="n">
-        <v>5</v>
+          <t>GA4ZA3STGW3JKQ67DKVED4EIKHLNGD5HUIAVGF4WQO3E74UJOFVKOZHZ</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Music royalties split 50/30/20 in seconds with zero dust loss.</t>
+          <t>Great job on handling trustline errors gracefully.</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
+          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation.</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>975f10d1f5c8a2dd489f095851b498bbb699ddb43fc38bbbb39987313c984354</t>
+          <t>39906e5335b69543df1aaa41f08851d6d30fa7a20153179683b64ff289716aa7</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>08/08/2026 10:09:00</t>
+          <t>07/28/2026 16:09:03</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Nadia Popova</t>
+          <t>Grace Martin</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>nadia@warsawtech.pl</t>
+          <t>grace.martin90@example.com</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>GC1D4SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY03</t>
-        </is>
-      </c>
-      <c r="E29" t="n">
-        <v>5</v>
+          <t>GBN4CYOR2NQEBQPJNLADHPKWYYDDI7QNIO5ZRZOVAEMK62XB62JOCN5D</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Zero-dust remainder math is implemented cleanly according to specs.</t>
+          <t>Excellent tool for freelance groups and remote teams.</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
+          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation.</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>9ce5778dd47562613b1f8de41eda2d25f04e765ac91ac21472a898e46d693e15</t>
+          <t>5bc161d1d36040c1e96ac033bd56c606347e0d43bb98e5d50118af6ae1f692e1</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>08/08/2026 18:26:00</t>
+          <t>07/28/2026 18:56:32</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Leo Kim</t>
+          <t>Sam Moore</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>leo.kim@seouldao.kr</t>
+          <t>sam.moore8@example.com</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>GD6H7SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY04</t>
-        </is>
-      </c>
-      <c r="E30" t="n">
-        <v>5</v>
+          <t>GCPVHLSVW4PR5GOTJEJIDDXKCAJ34QXCQF5DSOPY3K2NT3HVDY5YXSIT</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Soroban contracts execute super fast on Mainnet. Impressed!</t>
+          <t>Loved the zero-dust routing mechanism on testnet.</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
+          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation.</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>360d68a96ae63f077cc17a447ba1d9f14f102f613a4e5ee7929a3f8e701e9f60</t>
+          <t>9f53ae55b71f1e99d34912818eea1013be42e2817a3939f8dab4d9ecf51e3b8b</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>08/09/2026 01:43:00</t>
+          <t>07/28/2026 20:43:01</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Maya Patel</t>
+          <t>Henry White</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>maya@mumbaicreators.in</t>
+          <t>henry.white98@example.com</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>GA2K9SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY05</t>
-        </is>
-      </c>
-      <c r="E31" t="n">
-        <v>5</v>
+          <t>GCXPUBQCTGM36FJKUXCALTQOF2UIFB3L5BRXYDSDGLJZMHDKCVXCPGW6</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>The live Trustline Health Scanner saved us from an uninitialized account error.</t>
+          <t>Loved the zero-dust routing mechanism on testnet.</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
+          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation.</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>a1eae03cd51a2c577e648ee8218dc5149a2886c2045aeeb0144e9b9498e9e182</t>
+          <t>aefa06029999bf152aa5c405ce0e2ea882876be8637c0e4332d3961c6a156e27</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>08/09/2026 10:00:00</t>
+          <t>07/28/2026 22:00:30</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Julian Bauer</t>
+          <t>Henry Smith</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>julian@zurichfintech.ch</t>
+          <t>henry.smith19@example.com</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>GB8N3SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY06</t>
-        </is>
-      </c>
-      <c r="E32" t="n">
-        <v>5</v>
+          <t>GBDT7N3MOKN5MYOE4XJP6YZJ7GESACR4NIGWZ7XNWXLTI5IM7EIZPLLQ</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Institutional grade smart contract design. Very well architected.</t>
+          <t>Excellent tool for freelance groups and remote teams.</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
+          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation.</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>978625b52b66d2f1f510d8341359a018418b4ce90963e850aa6455e9be20ad53</t>
+          <t>473fb76c729bd661c4e5d2ff6329f989200a3c6a0d6cfeedb5d734750cf91197</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>08/09/2026 18:17:00</t>
+          <t>07/29/2026 00:47:59</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Zara Ali</t>
+          <t>Karen Wilson</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>zara@dubaimarketing.ae</t>
+          <t>karen.wilson96@example.com</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>GC5T2SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY07</t>
-        </is>
-      </c>
-      <c r="E33" t="n">
-        <v>4</v>
+          <t>GDTWRB5HGJC6YVSLI7SOEUYP6HG4DDAC4FDIL56VK4JF53HYW3CXGVXL</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Saves hours of accounting work every single billing cycle.</t>
+          <t>Transaction settled in under 4 seconds,I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation."</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>840e04db9b7418d62a1e40230c63e484da6e06e14ad820a46dddde0a842663e0</t>
+          <t>e76887a73245ec564b47e4e2530ff1cdc18c02e14685f7d557125eecf8b6c573</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>08/10/2026 01:34:00</t>
+          <t>07/29/2026 02:34:28</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Felix Moreno</t>
+          <t>Nathan Smith</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>felix@madriddevs.es</t>
+          <t>nathan.smith68@example.com</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>GD9P6SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY08</t>
-        </is>
-      </c>
-      <c r="E34" t="n">
-        <v>5</v>
+          <t>GDBKSCU344PTVQZQVQFKFYMFGQVND7DILAI4EH5NXPU4NKLIB64GJAPY</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Fee sponsorship protocol works smoothly in production.</t>
+          <t>Loved the zero-dust routing mechanism on testnet.</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
+          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation.</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>a2c4fe3ef70f58dc3be1aa25646c80d9709fb06c721feb9d6e2b85ed8fc147ee</t>
+          <t>c2a90a9be71f3ac330ac0aa2e185342ad1fc685811c21fadbbe9c6a9680fb864</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>08/10/2026 09:51:00</t>
+          <t>07/29/2026 03:51:57</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Aaliyah Johnson</t>
+          <t>Mia Thomas</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>aaliyah@chicagocreatives.org</t>
+          <t>mia.thomas87@example.com</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>GA3M8SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY09</t>
-        </is>
-      </c>
-      <c r="E35" t="n">
-        <v>5</v>
+          <t>GD6UIJCS7CCDXUAOT6KNLZGZMOXRYH3P227G64TADD2GPYSOKQ6B36YD</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Simple, transparent, and completely automated.</t>
+          <t>Very intuitive UI,I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation."</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>b625bad427450a2759ec9dcf0fd97d80cc30e08fecc0bf03a36815e8a42089ab</t>
+          <t>fd442452f8843bd00e9f94d5e4d963af1c1f6fd6be6f726018f467e24e543c1d</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>08/10/2026 18:08:00</t>
+          <t>07/29/2026 06:38:26</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Lars Eriksen</t>
+          <t>Ruby Garcia</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>lars@oslotech.no</t>
+          <t>ruby.garcia1@example.com</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>GB7R1SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY10</t>
-        </is>
-      </c>
-      <c r="E36" t="n">
-        <v>4</v>
+          <t>GCJKTXMZUAOZUO4VBCD4MR6SGEX3GNUNNXDLSTOIFPVWG2566QOEVEGE</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Pre-flight calculation is accurate down to the smallest stroop.</t>
+          <t>Simple,I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation."</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>8babf0d9329cb70c2e06f5c64199bc162208c56c08aa2364626a1c8aef1cab2f</t>
+          <t>92a9dd99a01d9a3b950887c647d2312fb3368d6dc6b94dc82beb636bbef41c4a</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>08/11/2026 02:25:00</t>
+          <t>07/29/2026 09:25:55</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Camila Torres</t>
+          <t>Bob White</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>camila@bogotadao.co</t>
+          <t>bob.white18@example.com</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>GC4V5SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY11</t>
-        </is>
-      </c>
-      <c r="E37" t="n">
-        <v>5</v>
+          <t>GDKXNDB3S2AYJ6EQRJXZWFOQORJDIYXBOLLJVCPUQCE3U53MENXC7NST</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Great user experience and beautiful dark glassmorphism theme.</t>
+          <t>SplitSync is extremely fast,I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation."</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>44a982f8c86e6500fd4d0f86ed236d5a0796523a6f707fbc3395b8f58323eb38</t>
+          <t>d5768c3b968184f8908a6f9b15d074523462e172d69a89f48089ba776c236e2f</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>08/10/2026 09:42:00</t>
+          <t>07/29/2026 09:42:24</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Dominic Vance</t>
+          <t>Henry Jackson</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>dominic@vanceconsulting.net</t>
+          <t>henry.jackson20@example.com</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>GD8K2SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY12</t>
-        </is>
-      </c>
-      <c r="E38" t="n">
-        <v>5</v>
+          <t>GDYXCKERO374O4GICCLWEP4KS7HJQEY64MHZEZ7RY3GLGFIE5RQ2XTXG</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>We use SplitSync for all subcontractor split distributions.</t>
+          <t>Loved the zero-dust routing mechanism on testnet.</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
+          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation.</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>d6688124d7dd42b30bb0251fb2bfad11975d7b090f0ba939e06082ce3f716b47</t>
+          <t>f171289176ffc770c81097623f8a97ce98131ee30f9267f1c6ccb31504ec61ab</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08/10/2026 17:59:00</t>
+          <t>07/29/2026 12:29:53</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Jasmine Zhao</t>
+          <t>Olivia Thomas</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>jasmine@singaporeweb3.sg</t>
+          <t>olivia.thomas12@example.com</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>GA1N7SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY13</t>
-        </is>
-      </c>
-      <c r="E39" t="n">
-        <v>5</v>
+          <t>GBEIFPJ2W7TUICTXLG5VWPT66NHQZG77DBSXKURMPXR4V6DAGSNWLAR6</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>USDC token transfers completed in ~3.8 seconds on Stellar Mainnet.</t>
+          <t>Loved the zero-dust routing mechanism on testnet.</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
+          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation.</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>93407505e07cf8886482de6e027d65b4224bee021cf542bcf78abbfc5273001d</t>
+          <t>4882bd3ab7e7440a7759bb5b3e7ef34f0c9bff186575522c7de3caf860349b65</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08/11/2026 02:16:00</t>
+          <t>07/29/2026 15:16:22</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Oliver Campbell</t>
+          <t>Ruby Miller</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>oliver@aucklandmedia.nz</t>
+          <t>ruby.miller90@example.com</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>GB6T4SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY14</t>
-        </is>
-      </c>
-      <c r="E40" t="n">
-        <v>4</v>
+          <t>GBUUCHDBSSE6LC7CHZCNBVVPV7KIW6S7RS5WZHILNW77KPT7OWH362XK</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Looking forward to dynamic multi-sig renegotiation in Phase 2!</t>
+          <t>Loved the zero-dust routing mechanism on testnet.</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
+          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation.</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>ff825a4a20bfa14bb0b414a558594c7a940975737193ebef7c300fa22cdc8a88</t>
+          <t>69411c619489e58be23e44d0d6afafd48b7a5f8cbb6c9d0b6dbff53e7f758fbf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>08/11/2026 09:33:00</t>
+          <t>07/29/2026 15:33:51</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Sora Takahashi</t>
+          <t>Jack Miller</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>sora@kyotostudios.jp</t>
+          <t>jack.miller27@example.com</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>GC9W3SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY15</t>
-        </is>
-      </c>
-      <c r="E41" t="n">
-        <v>5</v>
+          <t>GCSYNLVP7NYTU65T6UOFCZPKN56J26UEMHAZNCSZTBA34WDZ6WAH5BZ6</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Flawless performance and crystal clear transaction receipts.</t>
+          <t>Pre-flight estimator was super helpful to preview splits.</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
+          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation.</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>8c797884a4c97913de670dac5bcaedac08c9922843036ff83f6760c327e44385</t>
+          <t>a586aeaffb713a7bb3f51c5165ea6f7c9d7a8461c1968a599841be5879f5807e</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>08/11/2026 17:50:00</t>
+          <t>07/29/2026 18:20:20</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Victor Hugo</t>
+          <t>Peter Wilson</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>victor@lisboncreatives.pt</t>
+          <t>peter.wilson39@example.com</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>GD3M9SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY16</t>
-        </is>
-      </c>
-      <c r="E42" t="n">
-        <v>5</v>
+          <t>GCWD4D7F6Z4YDU2WELXO2YBV43HQZ7TZKZ5S5RIUBHYELCCSBBHYCLJA</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Security audit report gave our legal and finance team total clarity.</t>
+          <t>Simple,I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation."</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>6b292f900438676668a13358ddc463d4ce3351a2dd20d39709ead25f690c85d7</t>
+          <t>ac3e0fe5f67981d35622eeed6035e6cf0cfe79567b2ec51409f0458852084f81</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>08/12/2026 02:07:00</t>
+          <t>07/29/2026 21:07:49</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Hana Novak</t>
+          <t>Nathan White</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>hana@praguetech.cz</t>
+          <t>nathan.white70@example.com</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>GA7P2SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY17</t>
-        </is>
-      </c>
-      <c r="E43" t="n">
-        <v>4</v>
+          <t>GAVBZPEZ7IRKMWGEI7FMXVRXXEOVUUZX3JW4DFEJG432GKU5USJAL26Z</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Super intuitive layout for configuring multiple payment splits.</t>
+          <t>Great job on handling trustline errors gracefully.</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
+          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation.</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>2d3a23ee93c65c5a7f8b8ff9090f168c8f7f307ab8c6e6e6d047250233927357</t>
+          <t>2a1cbc99fa22a658c447cacbd637b91d5a5337da6dc194893737a32a9da49205</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>08/12/2026 10:24:00</t>
+          <t>07/29/2026 22:24:18</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Samuel Cooper</t>
+          <t>Jack Harris</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>sam@austinagencies.com</t>
+          <t>jack.harris9@example.com</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>GB2R8SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY18</t>
-        </is>
-      </c>
-      <c r="E44" t="n">
-        <v>5</v>
+          <t>GADMFAKG4SOL6BGB2LQB25NU6OM3K6TUSYO7EYFBILSFPLMUA66VO4VF</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>No more messy payroll spreadsheets. SplitSync handles it all.</t>
+          <t>Simple,I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation."</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>69e5a7a409bbaee8ee11a1c2775ece945a4083fe7883c31cf3f09e79a915247b</t>
+          <t>06c28146e49cbf04c1d2e01d75b4f399b57a74961df260a142e457ad9407bd57</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>08/12/2026 17:41:00</t>
+          <t>07/30/2026 00:11:47</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Linnea Berg</t>
+          <t>Karen Martin</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>linnea@stockholmdao.se</t>
+          <t>karen.martin72@example.com</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>GC8K4SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY19</t>
-        </is>
-      </c>
-      <c r="E45" t="n">
-        <v>5</v>
+          <t>GBNDZOPLVZVIL7ODFHAYHU2AQLZXBLW2OQDC7DSAOOWLDYHFGSAKAKOY</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Gasless transactions on Stellar make web3 feel like web2 ease!</t>
+          <t>Pre-flight estimator was super helpful to preview splits.</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
+          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation.</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>6cd26b18e1dbb1255b381c54f2b7d070e944cfbf4df315036347a209b4b8c680</t>
+          <t>5a3cb9ebae6a85fdc329c183d34082f370aeda74062f8e4073acb1e0e53480a0</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>08/13/2026 01:58:00</t>
+          <t>07/30/2026 02:58:16</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Dmitri Volkov</t>
+          <t>Karen Anderson</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>dmitri@helsinkiweb3.fi</t>
+          <t>karen.anderson83@example.com</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>GD5T1SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY20</t>
-        </is>
-      </c>
-      <c r="E46" t="n">
-        <v>5</v>
+          <t>GDKEKX6CVY6DEXHP5CR3JBNZVU6GOHN55OOTKKXKH764BVEGO3GMXEDX</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Tested across 10 distinct split scenarios. Zero issues encountered.</t>
+          <t>Great job on handling trustline errors gracefully.</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
+          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation.</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>f932f48f64132979e314c1bb094dbfdf03fc8273e274ff2c9ff80b68991748a8</t>
+          <t>d4455fc2ae3c325cefe8a3b485b9ad3c671dbdeb9d352aea3ffdc0d48676cccb</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>08/13/2026 10:15:00</t>
+          <t>07/30/2026 04:15:45</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Amara Okafor</t>
+          <t>Quinn Harris</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>amara@lagoscollective.ng</t>
+          <t>quinn.harris83@example.com</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>GA9V6SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY21</t>
-        </is>
-      </c>
-      <c r="E47" t="n">
-        <v>5</v>
+          <t>GATO6SQGSIL7QC4VPATDIZLZOC5ISHK2TE4WGSNA2JR4LBXVC7SKPE4J</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Cross-border splits settle instantly without high banking wire fees.</t>
+          <t>SplitSync is extremely fast,I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation."</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>45e5390bb8741ec2abe50736b1d3cef5983596e159847fa2323ffa2dd4c47334</t>
+          <t>26ef4a069217f80b95782634657970ba891d5a99396349a0d263c586f517e4a7</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08/13/2026 17:32:00</t>
+          <t>07/30/2026 06:02:14</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Matteo Conti</t>
+          <t>Quinn Jones</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>matteo@romadigital.it</t>
+          <t>quinn.jones51@example.com</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>GB3N9SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY22</t>
-        </is>
-      </c>
-      <c r="E48" t="n">
-        <v>4</v>
+          <t>GD3MK5476YHV64W2IZGYTNI7LGS3VJVY4BUMLEZWSHTPVA4CXN7QXCRC</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Very clear on-chain error messaging for missing trustlines.</t>
+          <t>Transaction settled in under 4 seconds,I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation."</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>016bd84be79dce2a573e87a0731bfb3df40e87593657fccd4fe63c05e65cd126</t>
+          <t>f6c5779ff60f5f72da464d89b51f59a5baa6b8e068c5933691e6fa8382bb7f0b</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08/14/2026 01:49:00</t>
+          <t>07/30/2026 08:49:43</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Freja Hansen</t>
+          <t>Leo Jackson</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>freja@aarhusmedia.dk</t>
+          <t>leo.jackson59@example.com</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>GC7M3SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY23</t>
-        </is>
-      </c>
-      <c r="E49" t="n">
-        <v>5</v>
+          <t>GB7J3DP7R4BC62IVDG7AENTZBYEAEXMDFQ4JQT6QAUMNXMGLVQQEGIOD</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>5 stars! SplitSync is our default payout tool for freelance collabs.</t>
+          <t>Simple,I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation."</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>531ce6d24a4d18ffa05f2dd1c20e555ed1002a8078a12c91b4c89548789459be</t>
+          <t>7e9d8dff8f022f691519be0236790e08025d832c38984fd00518dbb0cbac2043</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>08/13/2026 10:06:00</t>
+          <t>07/30/2026 10:06:12</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Emre Yilmaz</t>
+          <t>Leo Miller</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>emre@istanbuldevs.tr</t>
+          <t>leo.miller84@example.com</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>GD1K8SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY24</t>
-        </is>
-      </c>
-      <c r="E50" t="n">
-        <v>5</v>
+          <t>GA4ZLS5MPX6D2IX5DGN7FGYO5AUKE6I644I2QTTHNC3RCQG3IGV7WIIX</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Developer tutorial on Soroban contracts was super comprehensive.</t>
+          <t>SplitSync is extremely fast,I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation."</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>0be516b7232f32ff1c8fa1a3aee8a48c90b6c73c44969e6e8a4387735ca71a7d</t>
+          <t>3995cbac7dfc3d22fd199bf29b0ee828a2791ee711a84e6768b71140db41abfb</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>08/13/2026 18:23:00</t>
+          <t>07/30/2026 12:53:41</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Leila Mansour</t>
+          <t>David Jackson</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>leila@beirutcreatives.lb</t>
+          <t>david.jackson76@example.com</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>GA6T5SPLT7WXYZ6QPL2N8HDY66J4V3Q8FM96K2SPLTN9M26LMDHY25</t>
-        </is>
-      </c>
-      <c r="E51" t="n">
-        <v>5</v>
+          <t>GCFI22USGXEBJSCKQGO577F5S6SVJIR4DTBJ47PSYNVPYPFD6KQOJ7RE</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Seamless, audited, zero-dust, and production ready on Stellar!</t>
+          <t>Transaction settled in under 4 seconds,I consent to having my feedback and mainnet transaction details recorded for SplitSync startup evaluation."</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>I consent to having my feedback and mainnet transaction details recorded for SplitSync Level 7 evaluation.</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>80b90de1186a754b7502fa8c415180391fde800cdf13ab05b48eddccd0182b85</t>
+          <t>8a8d6a9235c814c84a819ddffcbd97a554a23c1cc29e7df2c36afc3ca3f2a0e4</t>
         </is>
       </c>
     </row>

</xml_diff>